<commit_message>
Add biological insight statistics release
</commit_message>
<xml_diff>
--- a/data_files/core/pesticide_data.xlsx
+++ b/data_files/core/pesticide_data.xlsx
@@ -4170,7 +4170,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Peroxidases</t>
+          <t>Oxidoreductases</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -7046,7 +7046,7 @@
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>Peroxidases</t>
+          <t>Oxidoreductases</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -7102,7 +7102,7 @@
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>Peroxidases</t>
+          <t>Oxidoreductases</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -14798,12 +14798,12 @@
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>Peroxidases</t>
+          <t>Oxidoreductases</t>
         </is>
       </c>
       <c r="I293" t="inlineStr">
         <is>
-          <t>laccase</t>
+          <t>Laccase</t>
         </is>
       </c>
       <c r="J293" t="inlineStr"/>
@@ -25542,7 +25542,7 @@
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>Peroxidases</t>
+          <t>Oxidoreductases</t>
         </is>
       </c>
       <c r="I514" t="inlineStr">
@@ -27662,7 +27662,7 @@
       </c>
       <c r="H556" t="inlineStr">
         <is>
-          <t>Peroxidases</t>
+          <t>Oxidoreductases</t>
         </is>
       </c>
       <c r="I556" t="inlineStr">
@@ -27714,7 +27714,7 @@
       </c>
       <c r="H557" t="inlineStr">
         <is>
-          <t>Peroxidases</t>
+          <t>Oxidoreductases</t>
         </is>
       </c>
       <c r="I557" t="inlineStr">
@@ -31506,7 +31506,7 @@
       </c>
       <c r="H631" t="inlineStr">
         <is>
-          <t>Peroxidases</t>
+          <t>Oxidoreductases</t>
         </is>
       </c>
       <c r="I631" t="inlineStr">
@@ -31558,12 +31558,12 @@
       </c>
       <c r="H632" t="inlineStr">
         <is>
-          <t>Peroxidases</t>
+          <t>Oxidoreductases</t>
         </is>
       </c>
       <c r="I632" t="inlineStr">
         <is>
-          <t>laccase</t>
+          <t>Laccase</t>
         </is>
       </c>
       <c r="J632" t="inlineStr"/>
@@ -31746,7 +31746,7 @@
       </c>
       <c r="H636" t="inlineStr">
         <is>
-          <t>Peroxidases</t>
+          <t>Oxidoreductases</t>
         </is>
       </c>
       <c r="I636" t="inlineStr">
@@ -34774,7 +34774,7 @@
       </c>
       <c r="H698" t="inlineStr">
         <is>
-          <t>Peroxidases</t>
+          <t>Oxidoreductases</t>
         </is>
       </c>
       <c r="I698" t="inlineStr">
@@ -36858,7 +36858,7 @@
       </c>
       <c r="H739" t="inlineStr">
         <is>
-          <t>Peroxidases</t>
+          <t>Oxidoreductases</t>
         </is>
       </c>
       <c r="I739" t="inlineStr">
@@ -43518,7 +43518,7 @@
       </c>
       <c r="H870" t="inlineStr">
         <is>
-          <t>Peroxidases</t>
+          <t>Oxidoreductases</t>
         </is>
       </c>
       <c r="I870" t="inlineStr">
@@ -43678,7 +43678,7 @@
       </c>
       <c r="H873" t="inlineStr">
         <is>
-          <t>Peroxidases</t>
+          <t>Oxidoreductases</t>
         </is>
       </c>
       <c r="I873" t="inlineStr">
@@ -43838,7 +43838,7 @@
       </c>
       <c r="H876" t="inlineStr">
         <is>
-          <t>Peroxidases</t>
+          <t>Oxidoreductases</t>
         </is>
       </c>
       <c r="I876" t="inlineStr">
@@ -43942,7 +43942,7 @@
       </c>
       <c r="H878" t="inlineStr">
         <is>
-          <t>Peroxidases</t>
+          <t>Oxidoreductases</t>
         </is>
       </c>
       <c r="I878" t="inlineStr">

</xml_diff>